<commit_message>
graphs of community means x microclimatic gradients
</commit_message>
<xml_diff>
--- a/results/LM FD x microclimatic gradients.xlsx
+++ b/results/LM FD x microclimatic gradients.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\OneDrive - Universidad de Oviedo\IMIB\Softwares\GitHub\Germination_drivers\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unioviedo-my.sharepoint.com/personal/espinosaclara_uniovi_es/Documents/IMIB/Softwares/GitHub/Germination_drivers/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F59DE300-92A5-4975-93DE-3DB3F913E1A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{F59DE300-92A5-4975-93DE-3DB3F913E1A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9872DCE-DB66-48D6-8570-FE3DC5E8381E}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{E2F4E602-5982-49DE-AF44-84CAAD4FA04A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{E2F4E602-5982-49DE-AF44-84CAAD4FA04A}"/>
   </bookViews>
   <sheets>
     <sheet name="transformed variables" sheetId="2" r:id="rId1"/>
@@ -251,6 +251,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -698,59 +702,61 @@
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
     </row>
-    <row r="5" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B5" s="2"/>
-      <c r="C5" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="C5" s="2"/>
       <c r="D5" s="2"/>
-      <c r="E5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="I5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+    </row>
+    <row r="6" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="O5" s="2"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
+      <c r="C6" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
+      <c r="E6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="G6" s="2"/>
       <c r="I6" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
+      <c r="M6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -759,12 +765,10 @@
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
       <c r="I7" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J7" s="2"/>
-      <c r="K7" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="K7" s="2"/>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
@@ -867,74 +871,74 @@
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
     </row>
-    <row r="12" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B12" s="2"/>
-      <c r="C12" s="2" t="s">
-        <v>32</v>
-      </c>
+      <c r="C12" s="2"/>
       <c r="D12" s="2"/>
-      <c r="E12" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
       <c r="G12" s="2"/>
       <c r="I12" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>27</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
-      <c r="M12" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>34</v>
-      </c>
+      <c r="M12" s="2"/>
+      <c r="N12" s="2"/>
       <c r="O12" s="2"/>
     </row>
     <row r="13" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>27</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="B13" s="2"/>
       <c r="C13" s="2" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
+      <c r="E13" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="G13" s="2"/>
       <c r="I13" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="J13" s="2"/>
+        <v>3</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
+      <c r="M13" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="N13" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="O13" s="2"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
+        <v>4</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
       <c r="I14" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
@@ -953,7 +957,7 @@
     <mergeCell ref="J9:O9"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="87" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1092,55 +1096,55 @@
       </c>
       <c r="O4" s="2"/>
     </row>
-    <row r="5" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
-      <c r="F5" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="I5" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
-      <c r="M5" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
       <c r="O5" s="2"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
+      <c r="F6" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="G6" s="2"/>
       <c r="I6" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
+      <c r="M6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -1149,7 +1153,7 @@
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
       <c r="I7" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
@@ -1257,75 +1261,75 @@
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
     </row>
-    <row r="12" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
-      <c r="E12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
       <c r="G12" s="2"/>
       <c r="I12" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J12" s="2"/>
-      <c r="K12" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="K12" s="2"/>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
-      <c r="N12" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="N12" s="2"/>
       <c r="O12" s="2"/>
     </row>
     <row r="13" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B13" s="2"/>
-      <c r="C13" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="C13" s="2"/>
       <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
+      <c r="E13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="G13" s="2"/>
       <c r="I13" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="O13" s="2"/>
+    </row>
+    <row r="14" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>5</v>
-      </c>
       <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
+      <c r="C14" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
       <c r="I14" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
+      <c r="M14" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
     </row>

</xml_diff>